<commit_message>
Update CS 424 Horowitz Small Data Sample 1.xlsx
</commit_message>
<xml_diff>
--- a/Data/CS 424 Horowitz Small Data Sample 1.xlsx
+++ b/Data/CS 424 Horowitz Small Data Sample 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/14270eef50ba1d21/Documents/UIC MS CS/Fall 2026/CS 424 Visualization and Visual Analytics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/14270eef50ba1d21/Documents/UIC MS CS/Fall 2026/CS 424 Visualization and Visual Analytics/Project/First Assignment/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96FBF45D-447B-4D16-A313-2E824DE01F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{96FBF45D-447B-4D16-A313-2E824DE01F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D17A6A77-60B3-4283-9A07-BE2FA7AB48A8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F2737CC4-5166-4FC6-9FF5-41052819B65E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="25">
   <si>
     <t>Observation ID</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>Bus got added to Ventra App, 1 minute early once added to app</t>
+  </si>
+  <si>
+    <t>Grand and Kingsbury</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Bus Bunched, three buses one after another</t>
+  </si>
+  <si>
+    <t>Arrived on time. Previous bus for route arrived over 20 minutes prior</t>
   </si>
 </sst>
 </file>
@@ -483,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15F4CDB0-5A9D-4AAD-941B-C29AAEACCBF1}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -710,6 +722,111 @@
         <v>20</v>
       </c>
     </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <v>66</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="I7">
+        <v>21</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>66</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.73958333333333337</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>4</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>66</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.74861111111111112</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.74027777777777781</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>10</v>
+      </c>
+      <c r="K9" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>